<commit_message>
Fix methodology: add NL linearmodels cross-check scripts, correct NDBI spec to level+LDV, update dashboard
- Add src/regression/run_nl_twfe_pooled.py: linearmodels PanelOLS cross-check for NL pooled
  (replicates pyfixest primary using Delta log NL outcome, same FE + district-clustered SEs)
- Add src/regression/run_nl_twfe_by_state.py: same cross-check run per state
- Fix src/regression/run_ndbi_pooled.py: change outcome from Delta NDBI to NDBI level with LDV
  (now matches pyfixest primary spec per dissertation Eq 2)
- Fix src/regression/run_ndbi_by_state.py: same spec correction per state
- Regenerate all 4 linearmodels Excel output files; cross-check confirms pyfixest estimates
- dashboard/utils/data_loader.py: 4-spec mapping (NL OLS, NDBI OLS, NL TWFE, NDBI TWFE)
- dashboard/pages/3_Regression_Results.py: 4 spec options, primary/cross-check labels, corrected notes
- dashboard/pages/1_Overview.py: real-time Plotly 2x2 grid replacing static PNG
</commit_message>
<xml_diff>
--- a/outputs/tables/Regression_Results_NDBI_By_State.xlsx
+++ b/outputs/tables/Regression_Results_NDBI_By_State.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,21 +452,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Outcome: Delta NDBI = NDBI_t - NDBI_{t-1} (level change).</t>
+          <t>Outcome: NDBI_t (level; NDBI is bounded in [-1,1]).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lagged regressors: NDVI_{t-1}, NL_{t-1}. Seasonal_Ratio is contemporaneous.</t>
+          <t>Regressors: Seasonal_Ratio (contemp.), NDVI_{t-1}, NL_{t-1}, NDBI_{t-1} (lagged DV).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TWFE PanelOLS, AC + YEAR FE, SEs clustered by district (ST_CODE_DT_CODE).</t>
+          <t>TWFE PanelOLS (linearmodels), AC + YEAR FE, SEs clustered by district (ST_CODE_DT_CODE).</t>
         </is>
       </c>
     </row>
@@ -474,6 +474,20 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>Estimated separately for each state. Significance: *** p&lt;0.01, ** p&lt;0.05, * p&lt;0.10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nickell bias: lagged NDBI_{t-1} with entity FE biases its coefficient ~1/T ≈ 20%; flood coef far less affected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cross-check: same specification as run_ndbi_ols_by_state.py (pyfixest); coefficients should be close.</t>
         </is>
       </c>
     </row>
@@ -488,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -530,16 +544,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.1622200014101812</v>
+        <v>-0.08595938447122288</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05856516762206613</v>
+        <v>0.01662369642965734</v>
       </c>
       <c r="D2" t="n">
-        <v>-2.769905867204589</v>
+        <v>-5.170894742631842</v>
       </c>
       <c r="E2" t="n">
-        <v>0.005786512019847034</v>
+        <v>3.212251229456342e-07</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -554,16 +568,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.001948284705617928</v>
+        <v>0.01497373250925963</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01519134493749041</v>
+        <v>0.009755670464040075</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1282496522615188</v>
+        <v>1.53487477508118</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8979957867905624</v>
+        <v>0.1253598811459096</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -578,16 +592,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4565422891145278</v>
+        <v>0.1036360124422682</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1809115723559678</v>
+        <v>0.04856910403629649</v>
       </c>
       <c r="D4" t="n">
-        <v>2.523565978500366</v>
+        <v>2.133784727937731</v>
       </c>
       <c r="E4" t="n">
-        <v>0.011882666114851</v>
+        <v>0.03327927818893173</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -602,18 +616,42 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.002728775542155587</v>
+        <v>0.002214100649532697</v>
       </c>
       <c r="C5" t="n">
-        <v>0.002537920623606795</v>
+        <v>0.0007929652795989019</v>
       </c>
       <c r="D5" t="n">
-        <v>1.075201295412288</v>
+        <v>2.792178556232165</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2827309128839011</v>
+        <v>0.005408077380776533</v>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>p &lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NDBI_mean_t_minus_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.04681102681448827</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.03294339170724195</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-1.420953471654765</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.1558676788551152</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
@@ -630,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -672,20 +710,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.02267669845225912</v>
+        <v>-0.159832403523132</v>
       </c>
       <c r="C2" t="n">
-        <v>0.04489728002377091</v>
+        <v>0.01247137709288163</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.5050795602818906</v>
+        <v>-12.81593863554656</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6135984870500175</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>n.s.</t>
+          <t>p &lt; 0.01</t>
         </is>
       </c>
     </row>
@@ -696,20 +734,20 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.04433060884454944</v>
+        <v>0.01036354133839794</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01678809310514855</v>
+        <v>0.01389752847063237</v>
       </c>
       <c r="D3" t="n">
-        <v>-2.640598224401924</v>
+        <v>0.7457111068559932</v>
       </c>
       <c r="E3" t="n">
-        <v>0.008386639876435842</v>
+        <v>0.4559925064974966</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -720,16 +758,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1443268224738918</v>
+        <v>-0.01110018519866909</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1426889468181347</v>
+        <v>0.02896896514108791</v>
       </c>
       <c r="D4" t="n">
-        <v>1.011478644227745</v>
+        <v>-0.3831750683743006</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3119974223231434</v>
+        <v>0.7016599282894522</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -744,20 +782,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.002418610053482274</v>
+        <v>0.0007431473913349661</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005735852900434005</v>
+        <v>0.000297563995526686</v>
       </c>
       <c r="D5" t="n">
-        <v>-4.216652859593505</v>
+        <v>2.497437198407021</v>
       </c>
       <c r="E5" t="n">
-        <v>2.671558869993262e-05</v>
+        <v>0.01264670986094307</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>p &lt; 0.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NDBI_mean_t_minus_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.01940452175475877</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.05205505728728561</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.3727691941182111</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.7093880978290348</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -836,7 +898,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4076262703419949</v>
+        <v>-0.07382871089116483</v>
       </c>
     </row>
     <row r="3">
@@ -863,7 +925,7 @@
         <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>0.414959515921527</v>
+        <v>-0.06897133896329111</v>
       </c>
     </row>
   </sheetData>
@@ -941,7 +1003,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1606522740196467</v>
+        <v>0.1037380333373623</v>
       </c>
     </row>
     <row r="3">
@@ -968,7 +1030,7 @@
         <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1331746999012206</v>
+        <v>0.09181417071592501</v>
       </c>
     </row>
   </sheetData>
@@ -1046,7 +1108,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.004828943163594834</v>
+        <v>-0.09577252478147824</v>
       </c>
     </row>
     <row r="3">
@@ -1073,7 +1135,7 @@
         <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.01278038753847532</v>
+        <v>-0.09981811964314935</v>
       </c>
     </row>
   </sheetData>
@@ -1151,7 +1213,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1304863665283108</v>
+        <v>-0.002355451884639148</v>
       </c>
     </row>
     <row r="3">
@@ -1178,7 +1240,7 @@
         <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>0.08258265489110272</v>
+        <v>-7.660042303347936e-06</v>
       </c>
     </row>
   </sheetData>
@@ -1192,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1269,10 +1331,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.4693765780662719</v>
+        <v>-0.3234905274800184</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02744477096722257</v>
+        <v>0.01978721008847815</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1280,21 +1342,21 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-0.08418572321153393</v>
+        <v>0.09377105846868268</v>
       </c>
       <c r="F2" t="n">
-        <v>0.05099280346339597</v>
+        <v>0.03520501373518449</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>p &lt; 0.10</t>
+          <t>p &lt; 0.01</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>-0.2436553522025553</v>
+        <v>-0.06933492829310611</v>
       </c>
       <c r="I2" t="n">
-        <v>0.06768253447196962</v>
+        <v>0.02304861334245618</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -1302,14 +1364,14 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>-0.07629404101824984</v>
+        <v>-0.1486782956904094</v>
       </c>
       <c r="L2" t="n">
-        <v>0.046796118840222</v>
+        <v>0.01530079411967304</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>n.s.</t>
+          <t>p &lt; 0.01</t>
         </is>
       </c>
     </row>
@@ -1320,10 +1382,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.02961945076132502</v>
+        <v>-0.02343934171717115</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00939625753667256</v>
+        <v>0.007885848513935425</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1331,10 +1393,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-0.07521046741516647</v>
+        <v>-0.05242179835305426</v>
       </c>
       <c r="F3" t="n">
-        <v>0.04595341836048673</v>
+        <v>0.0322866147248804</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1342,10 +1404,10 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.002847900279419802</v>
+        <v>0.01915160185997972</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01526650697151583</v>
+        <v>0.01170842137218953</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -1353,14 +1415,14 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>-0.04818264053539471</v>
+        <v>0.01006969119001572</v>
       </c>
       <c r="L3" t="n">
-        <v>0.01683915856034237</v>
+        <v>0.01745185241095015</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -1371,10 +1433,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.109864636773964</v>
+        <v>0.3456545325073494</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06387816005877185</v>
+        <v>0.07306254036123862</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1382,10 +1444,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.4061485282397764</v>
+        <v>-0.2075807322053122</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1232566486727815</v>
+        <v>0.06942677307064027</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1393,25 +1455,25 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.7078335707975628</v>
+        <v>0.1269780347618348</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2069409877783767</v>
+        <v>0.06741550121360265</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>p &lt; 0.10</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>0.3122563332346709</v>
+        <v>-0.01493468122104172</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1412726393106175</v>
+        <v>0.03607663998127501</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>p &lt; 0.05</t>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -1422,10 +1484,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.006492685104606586</v>
+        <v>0.005909806659476958</v>
       </c>
       <c r="C5" t="n">
-        <v>0.000936068706904669</v>
+        <v>0.0009777973510612529</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1433,89 +1495,113 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.006382178373274645</v>
+        <v>0.0007089535215174528</v>
       </c>
       <c r="F5" t="n">
-        <v>0.001577399245289156</v>
+        <v>0.0005316912745770792</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>n.s.</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.006024803233105602</v>
+        <v>0.003121466949012797</v>
       </c>
       <c r="I5" t="n">
-        <v>0.003072982163954998</v>
+        <v>0.001119411919125033</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>p &lt; 0.01</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.0006910278373330032</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0003894545761870442</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>p &lt; 0.10</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>-0.002196179401249924</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.0006628294551448594</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>p &lt; 0.01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Observations</t>
+          <t>NDBI_median_t_minus_1</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1215</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+        <v>0.108102881834785</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0665207420977544</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
+        </is>
+      </c>
       <c r="E6" t="n">
-        <v>475</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+        <v>0.02645027387081571</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.04940779151585706</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
+        </is>
+      </c>
       <c r="H6" t="n">
-        <v>735</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+        <v>-0.0287924628080574</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.04361877446649384</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
+        </is>
+      </c>
       <c r="K6" t="n">
-        <v>1465</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+        <v>0.0146349749074232</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.04815505968857339</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ACs (entities)</t>
+          <t>Observations</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>243</v>
+        <v>1215</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>81</v>
+        <v>475</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>147</v>
+        <v>735</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>293</v>
+        <v>1465</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
@@ -1523,26 +1609,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Districts (clusters)</t>
+          <t>ACs (entities)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>37</v>
+        <v>243</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>30</v>
+        <v>147</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>19</v>
+        <v>293</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
@@ -1550,26 +1636,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Years</t>
+          <t>Districts (clusters)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
@@ -1577,29 +1663,56 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>R-sq (within)</t>
+          <t>Years</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.4076262703419949</v>
+        <v>5</v>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>0.1606522740196467</v>
+        <v>5</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>0.004828943163594834</v>
+        <v>5</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>0.1304863665283108</v>
+        <v>5</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>R-sq (within)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.07382871089116483</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>0.1037380333373623</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>-0.09577252478147824</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>-0.002355451884639148</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1612,7 +1725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1654,13 +1767,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.4693765780662719</v>
+        <v>-0.3234905274800184</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02744477096722257</v>
+        <v>0.01978721008847815</v>
       </c>
       <c r="D2" t="n">
-        <v>-17.10258681432798</v>
+        <v>-16.34846580359416</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1678,16 +1791,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.02961945076132502</v>
+        <v>-0.02343934171717115</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00939625753667256</v>
+        <v>0.007885848513935425</v>
       </c>
       <c r="D3" t="n">
-        <v>-3.152260423442371</v>
+        <v>-2.972329696132316</v>
       </c>
       <c r="E3" t="n">
-        <v>0.001670107047635483</v>
+        <v>0.003028947331019882</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1702,16 +1815,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.109864636773964</v>
+        <v>0.3456545325073494</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06387816005877185</v>
+        <v>0.07306254036123862</v>
       </c>
       <c r="D4" t="n">
-        <v>17.37471204168718</v>
+        <v>4.730940517512134</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>2.568657282431275e-06</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1726,20 +1839,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.006492685104606586</v>
+        <v>0.005909806659476958</v>
       </c>
       <c r="C5" t="n">
-        <v>0.000936068706904669</v>
+        <v>0.0009777973510612529</v>
       </c>
       <c r="D5" t="n">
-        <v>6.936120240656452</v>
+        <v>6.043999457620484</v>
       </c>
       <c r="E5" t="n">
-        <v>7.37676586481939e-12</v>
+        <v>2.146158806226595e-09</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>p &lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NDBI_median_t_minus_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.108102881834785</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0665207420977544</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.625100358560707</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.1044680444241222</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1796,20 +1933,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.08418572321153393</v>
+        <v>0.09377105846868268</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05099280346339597</v>
+        <v>0.03520501373518449</v>
       </c>
       <c r="D2" t="n">
-        <v>-1.650933415966525</v>
+        <v>2.663571137169201</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0995633942267915</v>
+        <v>0.00805541145556421</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>p &lt; 0.10</t>
+          <t>p &lt; 0.01</t>
         </is>
       </c>
     </row>
@@ -1820,16 +1957,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.07521046741516647</v>
+        <v>-0.05242179835305426</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04595341836048673</v>
+        <v>0.0322866147248804</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.636667523298692</v>
+        <v>-1.623638736973483</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1025128610066421</v>
+        <v>0.1052692480630646</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1844,16 +1981,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4061485282397764</v>
+        <v>-0.2075807322053122</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1232566486727815</v>
+        <v>0.06942677307064027</v>
       </c>
       <c r="D4" t="n">
-        <v>3.295144989038351</v>
+        <v>-2.989923382930432</v>
       </c>
       <c r="E4" t="n">
-        <v>0.001074454212686593</v>
+        <v>0.002969239112883937</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1868,20 +2005,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.006382178373274645</v>
+        <v>0.0007089535215174528</v>
       </c>
       <c r="C5" t="n">
-        <v>0.001577399245289156</v>
+        <v>0.0005316912745770792</v>
       </c>
       <c r="D5" t="n">
-        <v>4.046013330065158</v>
+        <v>1.333393184007717</v>
       </c>
       <c r="E5" t="n">
-        <v>6.291484639642242e-05</v>
+        <v>0.1831891463671056</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>n.s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NDBI_median_t_minus_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.02645027387081571</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.04940779151585706</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.5353462087518464</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5927187663428044</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -1896,7 +2057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1938,16 +2099,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.2436553522025553</v>
+        <v>-0.06933492829310611</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06768253447196962</v>
+        <v>0.02304861334245618</v>
       </c>
       <c r="D2" t="n">
-        <v>-3.599973820476004</v>
+        <v>-3.008203889011807</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003454394796416072</v>
+        <v>0.002741942061141422</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1962,16 +2123,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.002847900279419802</v>
+        <v>0.01915160185997972</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01526650697151583</v>
+        <v>0.01170842137218953</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1865456377633338</v>
+        <v>1.635711702815004</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8520820098740867</v>
+        <v>0.1024424586682302</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1986,20 +2147,20 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7078335707975628</v>
+        <v>0.1269780347618348</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2069409877783767</v>
+        <v>0.06741550121360265</v>
       </c>
       <c r="D4" t="n">
-        <v>3.420460965208191</v>
+        <v>1.88351391706651</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0006690316450512768</v>
+        <v>0.06013081242116436</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>p &lt; 0.10</t>
         </is>
       </c>
     </row>
@@ -2010,20 +2171,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.006024803233105602</v>
+        <v>0.003121466949012797</v>
       </c>
       <c r="C5" t="n">
-        <v>0.003072982163954998</v>
+        <v>0.001119411919125033</v>
       </c>
       <c r="D5" t="n">
-        <v>1.960572145121579</v>
+        <v>2.788488219289849</v>
       </c>
       <c r="E5" t="n">
-        <v>0.05040635448241848</v>
+        <v>0.005469238100037188</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>p &lt; 0.10</t>
+          <t>p &lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NDBI_median_t_minus_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.0287924628080574</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.04361877446649384</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.660093346505519</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5094559731620492</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2080,20 +2265,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.07629404101824984</v>
+        <v>-0.1486782956904094</v>
       </c>
       <c r="C2" t="n">
-        <v>0.046796118840222</v>
+        <v>0.01530079411967304</v>
       </c>
       <c r="D2" t="n">
-        <v>-1.630349757823803</v>
+        <v>-9.717031320566941</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1032979038073147</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>n.s.</t>
+          <t>p &lt; 0.01</t>
         </is>
       </c>
     </row>
@@ -2104,20 +2289,20 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.04818264053539471</v>
+        <v>0.01006969119001572</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01683915856034237</v>
+        <v>0.01745185241095015</v>
       </c>
       <c r="D3" t="n">
-        <v>-2.861344904065982</v>
+        <v>0.5769984155777932</v>
       </c>
       <c r="E3" t="n">
-        <v>0.004293878897308145</v>
+        <v>0.5640520969482417</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -2128,20 +2313,20 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3122563332346709</v>
+        <v>-0.01493468122104172</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1412726393106175</v>
+        <v>0.03607663998127501</v>
       </c>
       <c r="D4" t="n">
-        <v>2.210310041338649</v>
+        <v>-0.4139709581821733</v>
       </c>
       <c r="E4" t="n">
-        <v>0.02727744196874382</v>
+        <v>0.6789716408586548</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>p &lt; 0.05</t>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -2152,20 +2337,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.002196179401249924</v>
+        <v>0.0006910278373330032</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0006628294551448594</v>
+        <v>0.0003894545761870442</v>
       </c>
       <c r="D5" t="n">
-        <v>-3.313340081982258</v>
+        <v>1.774347714946664</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0009502207340832403</v>
+        <v>0.07626699540395721</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>p &lt; 0.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NDBI_median_t_minus_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.0146349749074232</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.04815505968857339</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.3039135451616085</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.7612480752932487</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2257,10 +2466,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.4236793136683353</v>
+        <v>-0.3007150262805668</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02721388807397359</v>
+        <v>0.01947616943065709</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2268,10 +2477,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-0.08006082861556989</v>
+        <v>0.0463181427877646</v>
       </c>
       <c r="F2" t="n">
-        <v>0.04268863949418616</v>
+        <v>0.02646690008528062</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2279,10 +2488,10 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>-0.1622200014101812</v>
+        <v>-0.08595938447122288</v>
       </c>
       <c r="I2" t="n">
-        <v>0.05856516762206613</v>
+        <v>0.01662369642965734</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2290,14 +2499,14 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>-0.02267669845225912</v>
+        <v>-0.159832403523132</v>
       </c>
       <c r="L2" t="n">
-        <v>0.04489728002377091</v>
+        <v>0.01247137709288163</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>n.s.</t>
+          <t>p &lt; 0.01</t>
         </is>
       </c>
     </row>
@@ -2308,10 +2517,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.02762266211346719</v>
+        <v>-0.0211243078441686</v>
       </c>
       <c r="C3" t="n">
-        <v>0.007280858037810967</v>
+        <v>0.006654708884525821</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2319,10 +2528,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-0.05680349950899349</v>
+        <v>-0.04190856084311786</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03839191576137499</v>
+        <v>0.02687159585427024</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2330,10 +2539,10 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.001948284705617928</v>
+        <v>0.01497373250925963</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01519134493749041</v>
+        <v>0.009755670464040075</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2341,14 +2550,14 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>-0.04433060884454944</v>
+        <v>0.01036354133839794</v>
       </c>
       <c r="L3" t="n">
-        <v>0.01678809310514855</v>
+        <v>0.01389752847063237</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -2359,10 +2568,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.028430623221974</v>
+        <v>0.2820222565559276</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06476986931466158</v>
+        <v>0.06789361881045845</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2370,10 +2579,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.3467497382783501</v>
+        <v>-0.1417520317223072</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1067338887663635</v>
+        <v>0.05129314587897414</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2381,10 +2590,10 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.4565422891145278</v>
+        <v>0.1036360124422682</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1809115723559678</v>
+        <v>0.04856910403629649</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -2392,10 +2601,10 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>0.1443268224738918</v>
+        <v>-0.01110018519866909</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1426889468181347</v>
+        <v>0.02896896514108791</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -2410,10 +2619,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0056768233786671</v>
+        <v>0.004991720654479265</v>
       </c>
       <c r="C5" t="n">
-        <v>0.001214747154844553</v>
+        <v>0.0008456428203032133</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2421,89 +2630,113 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.004654527364931832</v>
+        <v>0.00066784766866399</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0005572054192816419</v>
+        <v>0.0003792202261518741</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>p &lt; 0.10</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.002728775542155587</v>
+        <v>0.002214100649532697</v>
       </c>
       <c r="I5" t="n">
-        <v>0.002537920623606795</v>
+        <v>0.0007929652795989019</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>n.s.</t>
+          <t>p &lt; 0.01</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>-0.002418610053482274</v>
+        <v>0.0007431473913349661</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0005735852900434005</v>
+        <v>0.000297563995526686</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>p &lt; 0.05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Observations</t>
+          <t>NDBI_mean_t_minus_1</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1215</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+        <v>0.05097985046341231</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0659050008630347</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
+        </is>
+      </c>
       <c r="E6" t="n">
-        <v>475</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+        <v>0.0860718586636931</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.03713077799928997</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>p &lt; 0.05</t>
+        </is>
+      </c>
       <c r="H6" t="n">
-        <v>735</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+        <v>-0.04681102681448827</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.03294339170724195</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
+        </is>
+      </c>
       <c r="K6" t="n">
-        <v>1465</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+        <v>0.01940452175475877</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.05205505728728561</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ACs (entities)</t>
+          <t>Observations</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>243</v>
+        <v>1215</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>81</v>
+        <v>475</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>147</v>
+        <v>735</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>293</v>
+        <v>1465</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
@@ -2511,26 +2744,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Districts (clusters)</t>
+          <t>ACs (entities)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>37</v>
+        <v>243</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>30</v>
+        <v>147</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>19</v>
+        <v>293</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
@@ -2538,26 +2771,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Years</t>
+          <t>Districts (clusters)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
@@ -2565,29 +2798,56 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>R-sq (within)</t>
+          <t>Years</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.414959515921527</v>
+        <v>5</v>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>0.1331746999012206</v>
+        <v>5</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>-0.01278038753847532</v>
+        <v>5</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>0.08258265489110272</v>
+        <v>5</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>R-sq (within)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.06897133896329111</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>0.09181417071592501</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>-0.09981811964314935</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>-7.660042303347936e-06</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2600,7 +2860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2642,13 +2902,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.4236793136683353</v>
+        <v>-0.3007150262805668</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02721388807397359</v>
+        <v>0.01947616943065709</v>
       </c>
       <c r="D2" t="n">
-        <v>-15.56849622210093</v>
+        <v>-15.44015250797812</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -2666,16 +2926,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.02762266211346719</v>
+        <v>-0.0211243078441686</v>
       </c>
       <c r="C3" t="n">
-        <v>0.007280858037810967</v>
+        <v>0.006654708884525821</v>
       </c>
       <c r="D3" t="n">
-        <v>-3.793874563961709</v>
+        <v>-3.174339886345578</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0001575461184268878</v>
+        <v>0.001549385007585835</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2690,16 +2950,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.028430623221974</v>
+        <v>0.2820222565559276</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06476986931466158</v>
+        <v>0.06789361881045845</v>
       </c>
       <c r="D4" t="n">
-        <v>15.87822600391096</v>
+        <v>4.153884584400506</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>3.558766952149739e-05</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2714,20 +2974,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0056768233786671</v>
+        <v>0.004991720654479265</v>
       </c>
       <c r="C5" t="n">
-        <v>0.001214747154844553</v>
+        <v>0.0008456428203032133</v>
       </c>
       <c r="D5" t="n">
-        <v>4.673255134640382</v>
+        <v>5.902871205941813</v>
       </c>
       <c r="E5" t="n">
-        <v>3.385440296765907e-06</v>
+        <v>4.944234577308748e-09</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>p &lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NDBI_mean_t_minus_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.05097985046341231</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0659050008630347</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.7735353887538794</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.439395234816742</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>n.s.</t>
         </is>
       </c>
     </row>
@@ -2742,7 +3026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2784,16 +3068,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.08006082861556989</v>
+        <v>0.0463181427877646</v>
       </c>
       <c r="C2" t="n">
-        <v>0.04268863949418616</v>
+        <v>0.02646690008528062</v>
       </c>
       <c r="D2" t="n">
-        <v>-1.875459831098002</v>
+        <v>1.750040338631274</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06148218090161639</v>
+        <v>0.08090591707978767</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2808,16 +3092,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.05680349950899349</v>
+        <v>-0.04190856084311786</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03839191576137499</v>
+        <v>0.02687159585427024</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.47956928906741</v>
+        <v>-1.559585856768461</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1398017658606774</v>
+        <v>0.1196772554108592</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2832,16 +3116,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3467497382783501</v>
+        <v>-0.1417520317223072</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1067338887663635</v>
+        <v>0.05129314587897414</v>
       </c>
       <c r="D4" t="n">
-        <v>3.248731422476064</v>
+        <v>-2.763566735734444</v>
       </c>
       <c r="E4" t="n">
-        <v>0.00126050267994593</v>
+        <v>0.005991177036704709</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2856,20 +3140,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.004654527364931832</v>
+        <v>0.00066784766866399</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005572054192816419</v>
+        <v>0.0003792202261518741</v>
       </c>
       <c r="D5" t="n">
-        <v>8.353341880508848</v>
+        <v>1.761107722130104</v>
       </c>
       <c r="E5" t="n">
-        <v>1.332267629550188e-15</v>
+        <v>0.07901190566673066</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>p &lt; 0.01</t>
+          <t>p &lt; 0.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NDBI_mean_t_minus_1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.0860718586636931</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.03713077799928997</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.318073126971349</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.02096734098803354</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>p &lt; 0.05</t>
         </is>
       </c>
     </row>

</xml_diff>